<commit_message>
Excel tools tracker: add Waves sheet + Wave 1 Status column to All Tools
- New 'Waves' sheet: Wave 1 branch summary (272 tools, 216P/13F/5Fi/38S)
- All Tools sheet: added 'Wave 1 Status' (col I) and 'Wave 1 Notes' (col J)
  - 272 tools colour-coded: green=Pass, red=Fail, yellow=Fishy, grey=Skip
  - 93 Category A tools (atf, incident, catalog etc.) left blank — not in Wave 1 scope

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solvvision/solvvision-mcp-tools.xlsx
+++ b/solvvision/solvvision-mcp-tools.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Tools" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Breakdown" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gaps" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="All Tools" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Waves" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="API Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gaps" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Tools'!$A$1:$H$366</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gaps'!$A$1:$C$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Gaps'!$A$1:$C$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +59,12 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +79,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C2410C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -120,6 +155,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -487,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H366"/>
+  <dimension ref="A1:J366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -498,6 +557,8 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -541,6 +602,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Wave 1 Status</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Wave 1 Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -579,6 +650,16 @@
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>Created STRY0010001 — cleanup needed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -617,6 +698,16 @@
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -659,6 +750,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>3 stories returned</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -697,6 +798,16 @@
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>Created EPIC0010001 — cleanup needed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -735,6 +846,16 @@
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -777,6 +898,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>3 epics returned</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -815,6 +946,16 @@
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>Created STSK0011002 — cleanup needed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -853,6 +994,16 @@
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -895,6 +1046,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>3 scrum tasks returned</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -937,6 +1098,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>3 apps returned (guard removed — was Phase 1 NOW_ASSIST-blocked)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -979,6 +1150,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake scope)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1017,6 +1198,16 @@
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` scope `x_wave1_grd_tst` — cleanup: `95131f3783280310ad3cc4d0deaad39a`</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1055,6 +1246,16 @@
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3201,6 +3402,16 @@
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
+      <c r="I67" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J67" s="13" t="inlineStr">
+        <is>
+          <t>Created CS0001002 — cleanup needed</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3243,6 +3454,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I68" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J68" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3281,6 +3502,16 @@
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
+      <c r="I69" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J69" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3323,6 +3554,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I70" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>3 cases returned</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3361,6 +3602,16 @@
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
+      <c r="I71" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J71" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3403,6 +3654,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I72" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J72" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3445,6 +3706,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I73" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J73" s="13" t="inlineStr">
+        <is>
+          <t>3 accounts returned</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3487,6 +3758,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I74" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J74" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3529,6 +3810,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I75" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J75" s="13" t="inlineStr">
+        <is>
+          <t>3 contacts returned</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3571,6 +3862,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I76" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J76" s="13" t="inlineStr">
+        <is>
+          <t>Empty results (no SLA on fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3613,6 +3914,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I77" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J77" s="13" t="inlineStr">
+        <is>
+          <t>3 products returned</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3655,6 +3966,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I78" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J78" s="13" t="inlineStr">
+        <is>
+          <t>Found `__guard_test__` script include by name pattern</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3693,6 +4014,16 @@
         </is>
       </c>
       <c r="H79" s="6" t="inlineStr"/>
+      <c r="I79" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J79" s="13" t="inlineStr">
+        <is>
+          <t>Validated `__guard_test__` script include — PASS, 0 issues</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3735,6 +4066,16 @@
           <t>multi-call: client.getRecord, client.createRecord</t>
         </is>
       </c>
+      <c r="I80" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J80" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id; requireScripting() succeeded)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3777,6 +4118,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I81" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J81" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake update_set_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3815,6 +4166,16 @@
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr"/>
+      <c r="I82" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J82" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake update_set_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3857,6 +4218,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I83" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J83" s="13" t="inlineStr">
+        <is>
+          <t>0 completed update sets in 7-day window</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3899,6 +4270,16 @@
           <t>Stub — returns placeholder; "Solution packaging requires Store app or manual export"</t>
         </is>
       </c>
+      <c r="I84" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J84" s="13" t="inlineStr">
+        <is>
+          <t>Returns message with update_set_count=1 (no API call)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3941,6 +4322,16 @@
           <t>generic dispatcher to Now Assist endpoints</t>
         </is>
       </c>
+      <c r="I85" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J85" s="13" t="inlineStr">
+        <is>
+          <t>Endpoint unavailable; caught gracefully (requireScripting() succeeded)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3979,6 +4370,16 @@
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr"/>
+      <c r="I86" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J86" s="13" t="inlineStr">
+        <is>
+          <t>Created `cmdb_ci` `__wave1_guard_test__` — cleanup: `4f64137b83280310ad3cc4d0deaad302`</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4021,6 +4422,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I87" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J87" s="13" t="inlineStr">
+        <is>
+          <t>Analyzed incident table — 1 stale, 1 empty assigned_to</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4063,6 +4474,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I88" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J88" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sn_devops_pipeline` — DevOps plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4101,6 +4522,16 @@
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr"/>
+      <c r="I89" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J89" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sn_devops_pipeline` — DevOps plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4143,6 +4574,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I90" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J90" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sn_devops_deploy_task` — DevOps plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4181,6 +4622,16 @@
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
+      <c r="I91" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J91" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sn_devops_deploy_task` — DevOps plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4219,6 +4670,16 @@
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr"/>
+      <c r="I92" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J92" s="13" t="inlineStr">
+        <is>
+          <t>Creates standard `change_request` (no DevOps plugin needed) — cleanup: `0af2973783280310ad3cc4d0deaad395` CHG0030059</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4257,6 +4718,16 @@
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
+      <c r="I93" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J93" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sn_devops_deploy_task` — DevOps plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4299,6 +4770,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I94" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J94" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sn_devops_deploy_task` — DevOps plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4341,6 +4822,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I95" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J95" s="13" t="inlineStr">
+        <is>
+          <t>3 flows returned</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4383,6 +4874,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I96" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J96" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4421,6 +4922,16 @@
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
+      <c r="I97" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J97" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INVALID_REQUEST: table `sys_hub_flow_trigger` does not exist; flows must be triggered via REST API — **escalate to Wave </t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4459,6 +4970,16 @@
         </is>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
+      <c r="I98" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J98" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4501,6 +5022,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I99" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J99" s="13" t="inlineStr">
+        <is>
+          <t>0 records (no executions for fake flow sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4543,6 +5074,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I100" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J100" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_hub_subflow` does not exist; subflows are stored in `sys_hub_flow` with `type=subflow` — **e</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4585,6 +5126,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I101" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J101" s="13" t="inlineStr">
+        <is>
+          <t>Same wrong table</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4627,6 +5178,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I102" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J102" s="13" t="inlineStr">
+        <is>
+          <t>3 action instances</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4669,6 +5230,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I103" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J103" s="13" t="inlineStr">
+        <is>
+          <t>`pa_process` table absent — PAD plugin not installed on PDI</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4711,6 +5282,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I104" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J104" s="13" t="inlineStr">
+        <is>
+          <t>`pa_process` table absent</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4749,6 +5330,16 @@
         </is>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
+      <c r="I105" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J105" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` flow — cleanup: `357e4f3783e40310ad3cc4d0deaad3b9`</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4787,6 +5378,16 @@
         </is>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
+      <c r="I106" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J106" s="13" t="inlineStr">
+        <is>
+          <t>Same wrong table `sys_hub_subflow`</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4825,6 +5426,16 @@
         </is>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
+      <c r="I107" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J107" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` action — cleanup: `d67e8f3783e40310ad3cc4d0deaad34d`</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4863,6 +5474,16 @@
         </is>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
+      <c r="I108" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J108" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id, guard removed)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4901,6 +5522,16 @@
         </is>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
+      <c r="I109" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J109" s="13" t="inlineStr">
+        <is>
+          <t>Same wrong table `sys_hub_flow_trigger`</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4943,6 +5574,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I110" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J110" s="13" t="inlineStr">
+        <is>
+          <t>0 records</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4981,6 +5622,16 @@
         </is>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
+      <c r="I111" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J111" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5023,6 +5674,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I112" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J112" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5061,6 +5722,16 @@
         </is>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
+      <c r="I113" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J113" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5103,6 +5774,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I114" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J114" s="13" t="inlineStr">
+        <is>
+          <t>Probe: INVALID_REQUEST sn_hr_core_case</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -5141,6 +5822,16 @@
         </is>
       </c>
       <c r="H115" s="6" t="inlineStr"/>
+      <c r="I115" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J115" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5183,6 +5874,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I116" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J116" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5225,6 +5926,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I117" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J117" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5267,6 +5978,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I118" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J118" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -5309,6 +6030,16 @@
           <t>multi-call: client.queryRecords, client.updateRecord</t>
         </is>
       </c>
+      <c r="I119" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J119" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5351,6 +6082,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I120" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J120" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -5389,6 +6130,16 @@
         </is>
       </c>
       <c r="H121" s="6" t="inlineStr"/>
+      <c r="I121" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J121" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -5431,6 +6182,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I122" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J122" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -5469,6 +6230,16 @@
         </is>
       </c>
       <c r="H123" s="6" t="inlineStr"/>
+      <c r="I123" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J123" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -5507,6 +6278,16 @@
         </is>
       </c>
       <c r="H124" s="6" t="inlineStr"/>
+      <c r="I124" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J124" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -5549,6 +6330,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I125" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J125" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -5591,6 +6382,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I126" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J126" s="13" t="inlineStr">
+        <is>
+          <t>HRSD plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -5903,6 +6704,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I134" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J134" s="13" t="inlineStr">
+        <is>
+          <t>3 REST messages returned</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -5945,6 +6756,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I135" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J135" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -5987,6 +6808,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I136" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J136" s="13" t="inlineStr">
+        <is>
+          <t>0 results (fake rest_message_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -6025,6 +6856,16 @@
         </is>
       </c>
       <c r="H137" s="6" t="inlineStr"/>
+      <c r="I137" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J137" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `3e9f8b3b83e40310ad3cc4d0deaad346`</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -6067,6 +6908,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I138" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J138" s="13" t="inlineStr">
+        <is>
+          <t>3 maps returned</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -6109,6 +6960,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I139" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J139" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -6147,6 +7008,16 @@
         </is>
       </c>
       <c r="H140" s="6" t="inlineStr"/>
+      <c r="I140" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J140" s="13" t="inlineStr">
+        <is>
+          <t>Created sys_import_set_run TH0001112 — cleanup: `df9f8b3b83e40310ad3cc4d0deaad3e8`</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -6189,6 +7060,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I141" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J141" s="13" t="inlineStr">
+        <is>
+          <t>0 results (fake transform_map_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -6231,6 +7112,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I142" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J142" s="13" t="inlineStr">
+        <is>
+          <t>3 import sets returned</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -6269,6 +7160,16 @@
         </is>
       </c>
       <c r="H143" s="6" t="inlineStr"/>
+      <c r="I143" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J143" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -6307,6 +7208,16 @@
         </is>
       </c>
       <c r="H144" s="6" t="inlineStr"/>
+      <c r="I144" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J144" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST (table doesn't exist) — guard removed</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -6349,6 +7260,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I145" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J145" s="13" t="inlineStr">
+        <is>
+          <t>3 data sources returned</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6391,6 +7312,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I146" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J146" s="13" t="inlineStr">
+        <is>
+          <t>3 events returned</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -6433,6 +7364,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I147" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ Fishy</t>
+        </is>
+      </c>
+      <c r="J147" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Query uses `name=` but field is `event_name` on sysevent_register; returns first record regardless of filter — escalate </t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -6471,6 +7412,16 @@
         </is>
       </c>
       <c r="H148" s="6" t="inlineStr"/>
+      <c r="I148" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ Fishy</t>
+        </is>
+      </c>
+      <c r="J148" s="13" t="inlineStr">
+        <is>
+          <t>SCRIPTING_ENABLED=true; record created but `event_name` is empty — code sets `name` instead of `event_name` — cleanup: `</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -6509,6 +7460,16 @@
         </is>
       </c>
       <c r="H149" s="6" t="inlineStr"/>
+      <c r="I149" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J149" s="13" t="inlineStr">
+        <is>
+          <t>Created sysevent record — cleanup: `d0afcb3b83e40310ad3cc4d0deaad3f9`</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -6551,6 +7512,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I150" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J150" s="13" t="inlineStr">
+        <is>
+          <t>3 heartbeat events returned</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -6593,6 +7564,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I151" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J151" s="13" t="inlineStr">
+        <is>
+          <t>3 OAuth apps returned</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -6635,6 +7616,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I152" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J152" s="13" t="inlineStr">
+        <is>
+          <t>3 aliases returned</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -6677,6 +7668,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I153" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J153" s="13" t="inlineStr">
+        <is>
+          <t>3 assets returned</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -6715,6 +7716,16 @@
         </is>
       </c>
       <c r="H154" s="6" t="inlineStr"/>
+      <c r="I154" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J154" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -6753,6 +7764,16 @@
         </is>
       </c>
       <c r="H155" s="6" t="inlineStr"/>
+      <c r="I155" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J155" s="13" t="inlineStr">
+        <is>
+          <t>Created `WAVE1-GUARD-TEST-001` — cleanup: `3dd2dff383280310ad3cc4d0deaad315`</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -6791,6 +7812,16 @@
         </is>
       </c>
       <c r="H156" s="6" t="inlineStr"/>
+      <c r="I156" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J156" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -6829,6 +7860,16 @@
         </is>
       </c>
       <c r="H157" s="6" t="inlineStr"/>
+      <c r="I157" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J157" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -6871,6 +7912,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I158" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J158" s="13" t="inlineStr">
+        <is>
+          <t>3 licenses returned</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -6913,6 +7964,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I159" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J159" s="13" t="inlineStr">
+        <is>
+          <t>36 licenses analyzed</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -6955,6 +8016,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I160" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J160" s="13" t="inlineStr">
+        <is>
+          <t>3 contracts returned</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -6997,6 +8068,16 @@
           <t>multi-call: client.queryRecords, client.updateRecord</t>
         </is>
       </c>
+      <c r="I161" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J161" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake asset_tag)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -7039,6 +8120,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I162" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J162" s="13" t="inlineStr">
+        <is>
+          <t>36 license recommendations returned</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -7363,6 +8454,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I170" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J170" s="13" t="inlineStr">
+        <is>
+          <t>Historical analysis returned (predicted_risk: low)</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -7405,6 +8506,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I171" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J171" s="13" t="inlineStr">
+        <is>
+          <t>0 anomalies in 3 incidents over 7 days</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -7447,6 +8558,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I172" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J172" s="13" t="inlineStr">
+        <is>
+          <t>Forecast returned (avg_daily_rate: 0.1)</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -7489,6 +8610,16 @@
           <t>multi-call: client.queryRecords, client.callNowAssist</t>
         </is>
       </c>
+      <c r="I173" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J173" s="13" t="inlineStr">
+        <is>
+          <t>PI solution found; training endpoint unavailable — returns training_failed gracefully</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -7531,6 +8662,16 @@
           <t>multi-call: client.queryRecords, client.callNowAssist</t>
         </is>
       </c>
+      <c r="I174" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J174" s="13" t="inlineStr">
+        <is>
+          <t>Same graceful failure path</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -7573,6 +8714,16 @@
           <t>Stub — returns placeholder; "Configure anomaly detection models via ML Workbench"</t>
         </is>
       </c>
+      <c r="I175" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J175" s="13" t="inlineStr">
+        <is>
+          <t>Returns queue message without API call</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -7611,6 +8762,16 @@
         </is>
       </c>
       <c r="H176" s="6" t="inlineStr"/>
+      <c r="I176" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J176" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake model_sys_id on ml_solution)</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -7653,6 +8814,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I177" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J177" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `ml_solution_version` does not exist — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -7695,6 +8866,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I178" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J178" s="13" t="inlineStr">
+        <is>
+          <t>0 conversations in 7-day window</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -7737,6 +8918,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I179" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J179" s="13" t="inlineStr">
+        <is>
+          <t>1 resolved incident analyzed, bottleneck LOW</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -7779,6 +8970,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I180" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J180" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_app_config` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -7817,6 +9018,16 @@
         </is>
       </c>
       <c r="H181" s="6" t="inlineStr"/>
+      <c r="I181" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J181" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_app_config` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -7855,6 +9066,16 @@
         </is>
       </c>
       <c r="H182" s="6" t="inlineStr"/>
+      <c r="I182" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J182" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_app_config` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -7897,6 +9118,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I183" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J183" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_applet` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -7935,6 +9166,16 @@
         </is>
       </c>
       <c r="H184" s="6" t="inlineStr"/>
+      <c r="I184" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J184" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_applet` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -7977,6 +9218,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I185" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J185" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_layout` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -8015,6 +9266,16 @@
         </is>
       </c>
       <c r="H186" s="6" t="inlineStr"/>
+      <c r="I186" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J186" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_layout` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -8053,6 +9314,16 @@
         </is>
       </c>
       <c r="H187" s="6" t="inlineStr"/>
+      <c r="I187" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J187" s="13" t="inlineStr">
+        <is>
+          <t>Created `sys_sg_offline_sync` record — cleanup: `dd441f3b83280310ad3cc4d0deaad3a5`</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -8091,6 +9362,16 @@
         </is>
       </c>
       <c r="H188" s="6" t="inlineStr"/>
+      <c r="I188" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J188" s="13" t="inlineStr">
+        <is>
+          <t>Created `sys_push_notification` record — cleanup: `21445f3b83280310ad3cc4d0deaad303`</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -8133,6 +9414,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I189" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J189" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_sg_mobile_session` — Mobile plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -8175,6 +9466,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I190" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J190" s="13" t="inlineStr">
+        <is>
+          <t>3 notifications returned</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -8217,6 +9518,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I191" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J191" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -8255,6 +9566,16 @@
         </is>
       </c>
       <c r="H192" s="6" t="inlineStr"/>
+      <c r="I192" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J192" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `cf0093bb83e40310ad3cc4d0deaad396`</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -8293,6 +9614,16 @@
         </is>
       </c>
       <c r="H193" s="6" t="inlineStr"/>
+      <c r="I193" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J193" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -8335,6 +9666,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I194" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J194" s="13" t="inlineStr">
+        <is>
+          <t>3 email log entries returned</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -8373,6 +9714,16 @@
         </is>
       </c>
       <c r="H195" s="6" t="inlineStr"/>
+      <c r="I195" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J195" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -8415,6 +9766,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I196" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J196" s="13" t="inlineStr">
+        <is>
+          <t>0 results (no attachments on fake record)</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -8453,6 +9814,16 @@
         </is>
       </c>
       <c r="H197" s="6" t="inlineStr"/>
+      <c r="I197" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J197" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake attachment_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -8491,6 +9862,16 @@
         </is>
       </c>
       <c r="H198" s="6" t="inlineStr"/>
+      <c r="I198" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J198" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake attachment_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -8533,6 +9914,16 @@
           <t>multipart upload, bypasses request() helper</t>
         </is>
       </c>
+      <c r="I199" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J199" s="13" t="inlineStr">
+        <is>
+          <t>Uploaded 4-byte txt — cleanup: `6c10d3bb83e40310ad3cc4d0deaad322`</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -8575,6 +9966,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I200" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J200" s="13" t="inlineStr">
+        <is>
+          <t>3 templates returned</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -8617,6 +10018,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I201" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J201" s="13" t="inlineStr">
+        <is>
+          <t>0 results</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -8655,6 +10066,16 @@
         </is>
       </c>
       <c r="H202" s="6" t="inlineStr"/>
+      <c r="I202" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J202" s="13" t="inlineStr">
+        <is>
+          <t>Created queued sys_email (fake recipient) — cleanup: `781017bb83e40310ad3cc4d0deaad338`</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -8693,6 +10114,16 @@
         </is>
       </c>
       <c r="H203" s="6" t="inlineStr"/>
+      <c r="I203" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J203" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake notification_id)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -9155,6 +10586,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I214" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J214" s="13" t="inlineStr">
+        <is>
+          <t>3 indicators returned</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -9197,6 +10638,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I215" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J215" s="13" t="inlineStr">
+        <is>
+          <t>Returned "% of incidents resolved by first assigned group"</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -9239,6 +10690,16 @@
           <t>multi-call: client.queryRecords, client.getRecord</t>
         </is>
       </c>
+      <c r="I216" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J216" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake indicator_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -9281,6 +10742,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I217" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J217" s="13" t="inlineStr">
+        <is>
+          <t>0 results (fake indicator_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -9323,6 +10794,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I218" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J218" s="13" t="inlineStr">
+        <is>
+          <t>3 breakdowns returned</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -9365,6 +10846,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I219" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J219" s="13" t="inlineStr">
+        <is>
+          <t>3 dashboards returned</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -9407,6 +10898,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I220" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J220" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -9449,6 +10950,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I221" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J221" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_ui_hp` does not exist — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -9491,6 +11002,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I222" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J222" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `pa_job` does not exist — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -9529,6 +11050,16 @@
         </is>
       </c>
       <c r="H223" s="6" t="inlineStr"/>
+      <c r="I223" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J223" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: same wrong table `pa_job`</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -9567,6 +11098,16 @@
         </is>
       </c>
       <c r="H224" s="6" t="inlineStr"/>
+      <c r="I224" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J224" s="13" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_PRIVILEGES — guard removed; PDI role limitation</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -9605,6 +11146,16 @@
         </is>
       </c>
       <c r="H225" s="6" t="inlineStr"/>
+      <c r="I225" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J225" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -9647,6 +11198,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I226" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J226" s="13" t="inlineStr">
+        <is>
+          <t>Analyzed incident (priority 100%, state 100%, assigned_to 90%)</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -9689,6 +11250,16 @@
           <t>multi-call: client.runAggregateQuery, client.queryRecords</t>
         </is>
       </c>
+      <c r="I227" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J227" s="13" t="inlineStr">
+        <is>
+          <t>81 incidents counted</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -9731,6 +11302,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I228" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J228" s="13" t="inlineStr">
+        <is>
+          <t>Returns counts for incident, change_request, problem</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -9773,6 +11354,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I229" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J229" s="13" t="inlineStr">
+        <is>
+          <t>3 portals returned</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -9811,6 +11402,16 @@
         </is>
       </c>
       <c r="H230" s="6" t="inlineStr"/>
+      <c r="I230" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J230" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `433f87f783e40310ad3cc4d0deaad32f`</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -9849,6 +11450,16 @@
         </is>
       </c>
       <c r="H231" s="6" t="inlineStr"/>
+      <c r="I231" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J231" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `a95f0ff783e40310ad3cc4d0deaad344`</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -9891,6 +11502,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I232" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J232" s="13" t="inlineStr">
+        <is>
+          <t>Returned "Service Portal" (url_suffix=sp)</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -9933,6 +11554,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I233" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ Fishy</t>
+        </is>
+      </c>
+      <c r="J233" s="13" t="inlineStr">
+        <is>
+          <t>50 records returned for newly-created empty portal; `sp_portal` filter on `sp_page` appears ignored — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -9971,6 +11602,16 @@
         </is>
       </c>
       <c r="H234" s="6" t="inlineStr"/>
+      <c r="I234" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J234" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -10013,6 +11654,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I235" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J235" s="13" t="inlineStr">
+        <is>
+          <t>3 widgets returned</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -10055,6 +11706,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I236" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J236" s="13" t="inlineStr">
+        <is>
+          <t>Returned "Cool Clock" widget by id</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -10093,6 +11754,16 @@
         </is>
       </c>
       <c r="H237" s="6" t="inlineStr"/>
+      <c r="I237" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J237" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `db3f87f783e40310ad3cc4d0deaad3aa`</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -10131,6 +11802,16 @@
         </is>
       </c>
       <c r="H238" s="6" t="inlineStr"/>
+      <c r="I238" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J238" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -10173,6 +11854,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I239" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J239" s="13" t="inlineStr">
+        <is>
+          <t>0 results (fake widget_sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -10215,6 +11906,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I240" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J240" s="13" t="inlineStr">
+        <is>
+          <t>3 UX apps returned</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -10257,6 +11958,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I241" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J241" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -10299,6 +12010,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I242" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ Fishy</t>
+        </is>
+      </c>
+      <c r="J242" s="13" t="inlineStr">
+        <is>
+          <t>22 records returned for fake app_sys_id; `ux_app_config` filter on `sys_ux_page` appears ignored — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -10341,6 +12062,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I243" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J243" s="13" t="inlineStr">
+        <is>
+          <t>3 themes returned</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -10379,6 +12110,16 @@
         </is>
       </c>
       <c r="H244" s="6" t="inlineStr"/>
+      <c r="I244" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J244" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -10577,6 +12318,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I249" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J249" s="13" t="inlineStr">
+        <is>
+          <t>3 reports returned</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -10619,6 +12370,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I250" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J250" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -10661,6 +12422,16 @@
           <t>aggregate counts grouped by field</t>
         </is>
       </c>
+      <c r="I251" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J251" s="13" t="inlineStr">
+        <is>
+          <t>5 priority groups returned for incident</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -10703,6 +12474,16 @@
           <t>aggregate counts grouped by field</t>
         </is>
       </c>
+      <c r="I252" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J252" s="13" t="inlineStr">
+        <is>
+          <t>2-month trend data returned</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -10745,6 +12526,16 @@
           <t>multi-call: client.callNowAssist, client.queryRecords</t>
         </is>
       </c>
+      <c r="I253" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J253" s="13" t="inlineStr">
+        <is>
+          <t>Fallback hits invalid table `pa_job_log` (INVALID_REQUEST) — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -10787,6 +12578,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I254" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J254" s="13" t="inlineStr">
+        <is>
+          <t>3 incidents exported</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -10829,6 +12630,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I255" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J255" s="13" t="inlineStr">
+        <is>
+          <t>QUERY_FAILED (syslog access restricted by role — not a guard error)</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -10871,6 +12682,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I256" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J256" s="13" t="inlineStr">
+        <is>
+          <t>3 jobs returned</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -10913,6 +12734,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I257" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J257" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake name)</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -10951,6 +12782,16 @@
         </is>
       </c>
       <c r="H258" s="6" t="inlineStr"/>
+      <c r="I258" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J258" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `ffa257f383280310ad3cc4d0deaad3a2`</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -10989,6 +12830,16 @@
         </is>
       </c>
       <c r="H259" s="6" t="inlineStr"/>
+      <c r="I259" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J259" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -11027,6 +12878,16 @@
         </is>
       </c>
       <c r="H260" s="6" t="inlineStr"/>
+      <c r="I260" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J260" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
@@ -11065,6 +12926,16 @@
         </is>
       </c>
       <c r="H261" s="6" t="inlineStr"/>
+      <c r="I261" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J261" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `54b297f383280310ad3cc4d0deaad330`</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -11103,6 +12974,16 @@
         </is>
       </c>
       <c r="H262" s="6" t="inlineStr"/>
+      <c r="I262" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J262" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
@@ -11145,6 +13026,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I263" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J263" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sysauto_trigger_log` does not exist — previously escalated to Wave 2 (Fix #10)</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -11183,6 +13074,16 @@
         </is>
       </c>
       <c r="H264" s="6" t="inlineStr"/>
+      <c r="I264" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J264" s="13" t="inlineStr">
+        <is>
+          <t>Created sysauto_report (Wave 1 fix verified) — cleanup: `e3b25bf383280310ad3cc4d0deaad3fa`</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -11221,6 +13122,16 @@
         </is>
       </c>
       <c r="H265" s="6" t="inlineStr"/>
+      <c r="I265" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J265" s="13" t="inlineStr">
+        <is>
+          <t>Created pa_indicators `__wave1_guard_test__` — cleanup: `b3b29bf383280310ad3cc4d0deaad302`</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -11263,6 +13174,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I266" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J266" s="13" t="inlineStr">
+        <is>
+          <t>Varun manual</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
@@ -11301,6 +13222,16 @@
         </is>
       </c>
       <c r="H267" s="6" t="inlineStr"/>
+      <c r="I267" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J267" s="13" t="inlineStr">
+        <is>
+          <t>Returned Auto assessment BR</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -11339,6 +13270,16 @@
         </is>
       </c>
       <c r="H268" s="6" t="inlineStr"/>
+      <c r="I268" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J268" s="13" t="inlineStr">
+        <is>
+          <t>Created `__guard_test__` — cleanup: `16db8bb383a40310ad3cc4d0deaad3e6`</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
@@ -11377,6 +13318,16 @@
         </is>
       </c>
       <c r="H269" s="6" t="inlineStr"/>
+      <c r="I269" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J269" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -11419,6 +13370,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I270" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J270" s="13" t="inlineStr">
+        <is>
+          <t>3 results returned</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
@@ -11461,6 +13422,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I271" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J271" s="13" t="inlineStr">
+        <is>
+          <t>Returned ComplianceCaseUtilsBase</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -11499,6 +13470,16 @@
         </is>
       </c>
       <c r="H272" s="6" t="inlineStr"/>
+      <c r="I272" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J272" s="13" t="inlineStr">
+        <is>
+          <t>Created `__guard_test__` — cleanup: `bedbcbb383a40310ad3cc4d0deaad3e2`</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -11537,6 +13518,16 @@
         </is>
       </c>
       <c r="H273" s="6" t="inlineStr"/>
+      <c r="I273" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J273" s="13" t="inlineStr">
+        <is>
+          <t>VALIDATION_ERROR (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -11579,6 +13570,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I274" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J274" s="13" t="inlineStr">
+        <is>
+          <t>1 result</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
@@ -11617,6 +13618,16 @@
         </is>
       </c>
       <c r="H275" s="6" t="inlineStr"/>
+      <c r="I275" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J275" s="13" t="inlineStr">
+        <is>
+          <t>Returned Autofill table name field</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
@@ -11659,6 +13670,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I276" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J276" s="13" t="inlineStr">
+        <is>
+          <t>1 result</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -11701,6 +13722,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I277" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J277" s="13" t="inlineStr">
+        <is>
+          <t>Returned IP Enrichment changeset</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -11739,6 +13770,16 @@
         </is>
       </c>
       <c r="H278" s="6" t="inlineStr"/>
+      <c r="I278" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J278" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -11777,6 +13818,16 @@
         </is>
       </c>
       <c r="H279" s="6" t="inlineStr"/>
+      <c r="I279" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J279" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -11815,6 +13866,16 @@
         </is>
       </c>
       <c r="H280" s="6" t="inlineStr"/>
+      <c r="I280" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J280" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `68dc47fb83640310ad3cc4d0deaad326`</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -11853,6 +13914,16 @@
         </is>
       </c>
       <c r="H281" s="6" t="inlineStr"/>
+      <c r="I281" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J281" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
@@ -11895,6 +13966,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I282" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J282" s="13" t="inlineStr">
+        <is>
+          <t>1 result</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -11933,6 +14014,16 @@
         </is>
       </c>
       <c r="H283" s="6" t="inlineStr"/>
+      <c r="I283" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J283" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
@@ -11971,6 +14062,16 @@
         </is>
       </c>
       <c r="H284" s="6" t="inlineStr"/>
+      <c r="I284" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J284" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `60dc07bb83a40310ad3cc4d0deaad309`</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -12013,6 +14114,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I285" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J285" s="13" t="inlineStr">
+        <is>
+          <t>1 result</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
@@ -12051,6 +14162,16 @@
         </is>
       </c>
       <c r="H286" s="6" t="inlineStr"/>
+      <c r="I286" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J286" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
@@ -12089,6 +14210,16 @@
         </is>
       </c>
       <c r="H287" s="6" t="inlineStr"/>
+      <c r="I287" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J287" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `b8dc07bb83a40310ad3cc4d0deaad39d`</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -12127,6 +14258,16 @@
         </is>
       </c>
       <c r="H288" s="6" t="inlineStr"/>
+      <c r="I288" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J288" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -12169,6 +14310,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I289" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J289" s="13" t="inlineStr">
+        <is>
+          <t>5 results on incident</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -12207,6 +14358,16 @@
         </is>
       </c>
       <c r="H290" s="6" t="inlineStr"/>
+      <c r="I290" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J290" s="13" t="inlineStr">
+        <is>
+          <t>Returned sn_customerservice_case.incident ACL</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
@@ -12245,6 +14406,16 @@
         </is>
       </c>
       <c r="H291" s="6" t="inlineStr"/>
+      <c r="I291" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J291" s="13" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_PRIVILEGES (guard removed, PDI role limit)</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
@@ -12283,6 +14454,16 @@
         </is>
       </c>
       <c r="H292" s="6" t="inlineStr"/>
+      <c r="I292" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J292" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
@@ -12321,6 +14502,16 @@
         </is>
       </c>
       <c r="H293" s="6" t="inlineStr"/>
+      <c r="I293" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J293" s="13" t="inlineStr">
+        <is>
+          <t>Created SIR0010002 — cleanup needed</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -12363,6 +14554,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I294" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J294" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
@@ -12401,6 +14602,16 @@
         </is>
       </c>
       <c r="H295" s="6" t="inlineStr"/>
+      <c r="I295" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J295" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
@@ -12443,6 +14654,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I296" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J296" s="13" t="inlineStr">
+        <is>
+          <t>3 SIR records</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -12485,6 +14706,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I297" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J297" s="13" t="inlineStr">
+        <is>
+          <t>3 CVE entries</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
@@ -12527,6 +14758,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I298" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J298" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
@@ -12565,6 +14806,16 @@
         </is>
       </c>
       <c r="H299" s="6" t="inlineStr"/>
+      <c r="I299" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J299" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
@@ -12607,6 +14858,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I300" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J300" s="13" t="inlineStr">
+        <is>
+          <t>3 risk records</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
@@ -12649,6 +14910,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I301" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J301" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
@@ -12691,6 +14962,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I302" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J302" s="13" t="inlineStr">
+        <is>
+          <t>3 controls</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
@@ -12733,6 +15014,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I303" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J303" s="13" t="inlineStr">
+        <is>
+          <t>3 IOC records</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
@@ -12775,6 +15066,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I304" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J304" s="13" t="inlineStr">
+        <is>
+          <t>sn_si_playbook table absent (partial SecOps plugin)</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
@@ -12813,6 +15114,16 @@
         </is>
       </c>
       <c r="H305" s="6" t="inlineStr"/>
+      <c r="I305" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J305" s="13" t="inlineStr">
+        <is>
+          <t>sn_si_playbook_execution table absent</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
@@ -12855,6 +15166,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I306" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J306" s="13" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_PRIVILEGES — guard removed; PDI role limit</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -12893,6 +15214,16 @@
         </is>
       </c>
       <c r="H307" s="6" t="inlineStr"/>
+      <c r="I307" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J307" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST from handler (ci_sys_ids required) — guard removed</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
@@ -12931,6 +15262,16 @@
         </is>
       </c>
       <c r="H308" s="6" t="inlineStr"/>
+      <c r="I308" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J308" s="13" t="inlineStr">
+        <is>
+          <t>Created RK0020248 — cleanup needed</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -12973,6 +15314,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I309" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J309" s="13" t="inlineStr">
+        <is>
+          <t>3 policies</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -13015,6 +15366,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I310" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J310" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST from handler (sys_id required) — guard removed</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
@@ -13057,6 +15418,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I311" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J311" s="13" t="inlineStr">
+        <is>
+          <t>sn_audit_result table absent (partial SecOps plugin)</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
@@ -13141,6 +15512,16 @@
           <t>multi-call: client.queryRecords, client.updateRecord, client.createRecord</t>
         </is>
       </c>
+      <c r="I313" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J313" s="13" t="inlineStr">
+        <is>
+          <t>Created `x.wave1.guard.test.1` — cleanup: `d1b0d73f83e40310ad3cc4d0deaad373`</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
@@ -13183,6 +15564,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I314" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J314" s="13" t="inlineStr">
+        <is>
+          <t>3 properties returned</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
@@ -13225,6 +15616,16 @@
           <t>multi-call: client.queryRecords, client.deleteRecord</t>
         </is>
       </c>
+      <c r="I315" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J315" s="13" t="inlineStr">
+        <is>
+          <t>`{deleted: false}` for nonexistent property</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
@@ -13267,6 +15668,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I316" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J316" s="13" t="inlineStr">
+        <is>
+          <t>3 glide.smtp results</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
@@ -13309,6 +15720,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I317" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J317" s="13" t="inlineStr">
+        <is>
+          <t>Both props not found on this PDI (correct)</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
@@ -13351,6 +15772,16 @@
           <t>multi-call: client.queryRecords, client.updateRecord, client.createRecord</t>
         </is>
       </c>
+      <c r="I318" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J318" s="13" t="inlineStr">
+        <is>
+          <t>Created `x.wave1.guard.test.2` — cleanup: name-based delete</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
@@ -13393,6 +15824,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I319" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ Fishy</t>
+        </is>
+      </c>
+      <c r="J319" s="13" t="inlineStr">
+        <is>
+          <t>category=email filter ignored; returned all 500 props (PDI has no categorized properties — query silently ignored) — esc</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -13435,6 +15876,16 @@
           <t>multi-call: client.queryRecords, client.updateRecord, client.createRecord</t>
         </is>
       </c>
+      <c r="I320" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J320" s="13" t="inlineStr">
+        <is>
+          <t>dry_run=true; showed "create" action (no writes)</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
@@ -13477,6 +15928,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I321" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J321" s="13" t="inlineStr">
+        <is>
+          <t>glide.smtp.host not found, returns "would be created as new"</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
@@ -13519,6 +15980,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I322" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J322" s="13" t="inlineStr">
+        <is>
+          <t>Only "(uncategorised)" category (998 records)</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
@@ -13561,6 +16032,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I323" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J323" s="13" t="inlineStr">
+        <is>
+          <t>3 audit history entries for glide.smtp.host</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
@@ -13763,6 +16244,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I328" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J328" s="13" t="inlineStr">
+        <is>
+          <t>5 in-progress update sets returned</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -13805,6 +16296,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I329" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J329" s="13" t="inlineStr">
+        <is>
+          <t>3 update sets returned</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
@@ -13847,6 +16348,16 @@
           <t>multi-call: client.createRecord, client.updateRecord</t>
         </is>
       </c>
+      <c r="I330" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J330" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` (switch_to=false) — cleanup: `05c09f3f83e40310ad3cc4d0deaad351`</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
@@ -13885,6 +16396,16 @@
         </is>
       </c>
       <c r="H331" s="6" t="inlineStr"/>
+      <c r="I331" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J331" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
@@ -13923,6 +16444,16 @@
         </is>
       </c>
       <c r="H332" s="6" t="inlineStr"/>
+      <c r="I332" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J332" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
@@ -13965,6 +16496,16 @@
           <t>multi-call: client.queryRecords, client.getRecord</t>
         </is>
       </c>
+      <c r="I333" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J333" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
@@ -14007,6 +16548,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I334" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J334" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
@@ -14049,6 +16600,16 @@
           <t>multi-call: client.queryRecords, client.createRecord</t>
         </is>
       </c>
+      <c r="I335" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J335" s="13" t="inlineStr">
+        <is>
+          <t>Found existing in-progress update set</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
@@ -14399,6 +16960,16 @@
         </is>
       </c>
       <c r="H344" s="6" t="inlineStr"/>
+      <c r="I344" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J344" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `61c09f3f83e40310ad3cc4d0deaad3ca`</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
@@ -14437,6 +17008,16 @@
         </is>
       </c>
       <c r="H345" s="6" t="inlineStr"/>
+      <c r="I345" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J345" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -14475,6 +17056,16 @@
         </is>
       </c>
       <c r="H346" s="6" t="inlineStr"/>
+      <c r="I346" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J346" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
@@ -14517,6 +17108,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I347" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J347" s="13" t="inlineStr">
+        <is>
+          <t>3 topics returned</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
@@ -14559,6 +17160,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I348" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J348" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_cs_conversation_message` does not exist — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
@@ -14601,6 +17212,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I349" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J349" s="13" t="inlineStr">
+        <is>
+          <t>0 results</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
@@ -14643,6 +17264,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I350" s="15" t="inlineStr">
+        <is>
+          <t>❌ Fail</t>
+        </is>
+      </c>
+      <c r="J350" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_cs_category` does not exist — escalate to Wave 2</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -14685,6 +17316,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I351" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J351" s="13" t="inlineStr">
+        <is>
+          <t>3 UIB pages returned</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
@@ -14723,6 +17364,16 @@
         </is>
       </c>
       <c r="H352" s="6" t="inlineStr"/>
+      <c r="I352" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J352" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
@@ -14761,6 +17412,16 @@
         </is>
       </c>
       <c r="H353" s="6" t="inlineStr"/>
+      <c r="I353" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J353" s="13" t="inlineStr">
+        <is>
+          <t>Created `__wave1_guard_test__` — cleanup: `b614173b83280310ad3cc4d0deaad32e`</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
@@ -14799,6 +17460,16 @@
         </is>
       </c>
       <c r="H354" s="6" t="inlineStr"/>
+      <c r="I354" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J354" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
@@ -14837,6 +17508,16 @@
         </is>
       </c>
       <c r="H355" s="6" t="inlineStr"/>
+      <c r="I355" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J355" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
@@ -14879,6 +17560,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I356" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J356" s="13" t="inlineStr">
+        <is>
+          <t>3 macroponents returned</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
@@ -14917,6 +17608,16 @@
         </is>
       </c>
       <c r="H357" s="6" t="inlineStr"/>
+      <c r="I357" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J357" s="13" t="inlineStr">
+        <is>
+          <t>Created `wave1-guard-test` — cleanup: `e714173b83280310ad3cc4d0deaad3ea`</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
@@ -14955,6 +17656,16 @@
         </is>
       </c>
       <c r="H358" s="6" t="inlineStr"/>
+      <c r="I358" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J358" s="13" t="inlineStr">
+        <is>
+          <t>NOT_FOUND (fake sys_id)</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
@@ -14997,6 +17708,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I359" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J359" s="13" t="inlineStr">
+        <is>
+          <t>3 data brokers returned</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
@@ -15035,6 +17756,16 @@
         </is>
       </c>
       <c r="H360" s="6" t="inlineStr"/>
+      <c r="I360" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J360" s="13" t="inlineStr">
+        <is>
+          <t>Created `wave1-guard-test` — cleanup: `a524973b83280310ad3cc4d0deaad39d`</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
@@ -15077,6 +17808,16 @@
           <t>table is parameterised by caller</t>
         </is>
       </c>
+      <c r="I361" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J361" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_aw_workspace` — Agent Workspace plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
@@ -15119,6 +17860,16 @@
           <t>multi-call: client.getRecord, client.queryRecords</t>
         </is>
       </c>
+      <c r="I362" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J362" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_aw_workspace` — Agent Workspace plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
@@ -15157,6 +17908,16 @@
         </is>
       </c>
       <c r="H363" s="6" t="inlineStr"/>
+      <c r="I363" s="14" t="inlineStr">
+        <is>
+          <t>⏭️ Skip</t>
+        </is>
+      </c>
+      <c r="J363" s="13" t="inlineStr">
+        <is>
+          <t>INVALID_REQUEST: table `sys_aw_workspace` — Agent Workspace plugin absent</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
@@ -15195,6 +17956,16 @@
         </is>
       </c>
       <c r="H364" s="6" t="inlineStr"/>
+      <c r="I364" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J364" s="13" t="inlineStr">
+        <is>
+          <t>Created `sys_aw_list` record — cleanup: `3124973b83280310ad3cc4d0deaad3dc`</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
@@ -15233,6 +18004,16 @@
         </is>
       </c>
       <c r="H365" s="6" t="inlineStr"/>
+      <c r="I365" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J365" s="13" t="inlineStr">
+        <is>
+          <t>Created `sys_ux_app_route` record — cleanup: `0a24973b83280310ad3cc4d0deaad3f4`</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
@@ -15271,6 +18052,16 @@
         </is>
       </c>
       <c r="H366" s="6" t="inlineStr"/>
+      <c r="I366" s="12" t="inlineStr">
+        <is>
+          <t>✅ Pass</t>
+        </is>
+      </c>
+      <c r="J366" s="13" t="inlineStr">
+        <is>
+          <t>Created `sys_ux_app_config` record — cleanup: `4224973b83280310ad3cc4d0deaad3ff`</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H366"/>
@@ -15279,6 +18070,159 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="54" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Wave</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Date Merged</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>Tools Tested</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>Fishy</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>Issue # Range</t>
+        </is>
+      </c>
+      <c r="K1" s="17" t="inlineStr">
+        <is>
+          <t>Fix Applied</t>
+        </is>
+      </c>
+      <c r="L1" s="17" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M1" s="17" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>wave-1-low-complexity-fixes</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>20 Category B handler files + reporting.ts</t>
+        </is>
+      </c>
+      <c r="E2" s="18" t="n">
+        <v>272</v>
+      </c>
+      <c r="F2" s="18" t="n">
+        <v>216</v>
+      </c>
+      <c r="G2" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="H2" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="18" t="n">
+        <v>38</v>
+      </c>
+      <c r="J2" s="18" t="inlineStr">
+        <is>
+          <t>#9 (fixed), #13–25 (escalated)</t>
+        </is>
+      </c>
+      <c r="K2" s="18" t="inlineStr">
+        <is>
+          <t>NOW_ASSIST guard bug fixed; table fixes for #7, #8, #9</t>
+        </is>
+      </c>
+      <c r="L2" s="18" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="M2" s="18" t="inlineStr">
+        <is>
+          <t>Skips: HRSD 16, Mobile 8, DevOps 6, Agent Workspace 3, SecOps-partial 3, PAD 2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15474,7 +18418,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>